<commit_message>
feat: add structural destruction and player camera
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2020,9 +2020,113 @@
       <c r="M29" s="3" t="inlineStr"/>
       <c r="N29" s="3" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Fracture and structural collapse</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Fire repeated Blast Charges or Concussion Grenades beneath an overhang</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Compare crater edges and watch the unsupported mass after supports are severed</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Blast edges vary deterministically and unsupported structural terrain cascades under gravity</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Short capture plus seed weapon and location</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="3" t="inlineStr"/>
+      <c r="N30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Player lock zoom and aim alignment</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Move P1 while changing 1x through 4x zoom with the mouse wheel</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Aim and fire at visible terrain at each zoom and frame cap</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Camera remains centered on P1 and reticle debug target and impact agree at every zoom</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Short capture plus zoom frame cap and impact location</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="3" t="inlineStr"/>
+      <c r="N31" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N29"/>
-  <conditionalFormatting sqref="H2:H29">
+  <autoFilter ref="A1:N31"/>
+  <conditionalFormatting sqref="H2:H31">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -2034,10 +2138,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: increase mini-voxel density tenfold
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2124,9 +2124,61 @@
       <c r="M31" s="3" t="inlineStr"/>
       <c r="N31" s="3" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Density</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Ten-times mini-voxel profile</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Start a seeded match and enable the debug overlay</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Inspect terrain particles explosions and the occupied-cell count</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>The demo uses a 256x160x10 world with granular terrain and effects at the denser scale</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot seed occupied count and benchmark output</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N31"/>
-  <conditionalFormatting sqref="H2:H31">
+  <autoFilter ref="A1:N32"/>
+  <conditionalFormatting sqref="H2:H32">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -2138,10 +2190,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: VOX DIGS v0.0.2 gamefeel demo
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -592,7 +592,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The VOX + DIGS title screen appears without an error</t>
+          <t>The DIGS title screen appears without an error</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -639,7 +639,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Cycle bots from 0 through 3; select each map style; change the seed; select each arsenal</t>
+          <t>Cycle local players from 1 through 2 and bots from 0 through 2; select each mode map style seed and arsenal</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Start a match with 1 to 3 bots</t>
+          <t>Start a match with 1 or 2 bots</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -2085,22 +2085,22 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Player lock zoom and aim alignment</t>
+          <t>Shared dynamic zoom and aim alignment</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Move P1 while changing 1x through 4x zoom with the mouse wheel</t>
+          <t>Start a two-human match and separate the players while changing zoom with the mouse wheel</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Aim and fire at visible terrain at each zoom and frame cap</t>
+          <t>Aim and fire at visible terrain from each local player at several frame caps</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Camera remains centered on P1 and reticle debug target and impact agree at every zoom</t>
+          <t>The spring camera keeps both humans readable; action weighting remains stable; and each reticle debug target and impact agree</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2176,9 +2176,1049 @@
       <c r="M32" s="3" t="inlineStr"/>
       <c r="N32" s="3" t="inlineStr"/>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Local Multiplayer</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>One and two human slot ownership</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Open Match Setup and cycle Local Players and Bots</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Start one-human plus bots and two-human plus bots matches</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Exactly four or fewer active slots are created; local inputs never drive bots; and both humans score die and respawn independently</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Setup screenshot and short capture from both match shapes</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr"/>
+      <c r="M33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Controller hotplug and Xbox layout</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Start with no controller then connect an Xbox-compatible controller</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Use the controller in menus and play; disconnect and reconnect it</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>The controller is claimed once; all documented actions work; disconnect pauses safely; and reconnect allows reclaim</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Controller model terminal output and short capture</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
+      <c r="M34" s="3" t="inlineStr"/>
+      <c r="N34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Responsive traversal game feel</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Use a flat recorded seed and then rough terrain</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Run reverse stop short-hop full-jump coyote jump-buffer and step-assist trials</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Acceleration is readable but responsive; reversal and stopping are precise; jump height responds to hold time; and small terrain steps do not dead-stop the miner</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Short capture with approximate flat-map traversal time</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr"/>
+      <c r="L35" s="3" t="inlineStr"/>
+      <c r="M35" s="3" t="inlineStr"/>
+      <c r="N35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Rope</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Deterministic breakable traversal rope</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Use visible beams arches and rock anchors</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Aim attach swing reel release and destroy the occupied anchor</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Rope attaches only to stable solids; constrains distance; preserves release momentum; and detaches safely when the anchor breaks</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Seed anchor location and short capture</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr"/>
+      <c r="L36" s="3" t="inlineStr"/>
+      <c r="M36" s="3" t="inlineStr"/>
+      <c r="N36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Spawn Safety</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Five-second spawn shield</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Start or respawn beside combat and hazards</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Observe 300 ticks; receive fire impulse and environmental contact; then make an offensive attack</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Shield blocks damage hostile impulse and environment harm for 300 ticks and ends early only on offensive use</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Debug tick capture showing spawn expiry and attack cancellation</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
+      <c r="M37" s="3" t="inlineStr"/>
+      <c r="N37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Weighted shared-camera momentum</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Play a two-human match with separation jumps ropes and nearby explosions</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Change direction quickly and trigger local and bot-only combat</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Camera uses smooth frame-rate-updated spring motion and subtle contextual zoom; local action affects it while distant bot-only events do not spam it</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>60 and 144 FPS matched captures</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
+      <c r="M38" s="3" t="inlineStr"/>
+      <c r="N38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Accessibility</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Flash gore shake and number controls</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Open Options and cycle Full Reduced Off variants plus damage-number settings</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Trigger local damage kills and explosions under each setting</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Feedback follows the selected setting; bot-only fights do not flash the screen; and presentation-only settings do not change authoritative simulation hashes</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Matched captures and hash notes</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
+      <c r="M39" s="3" t="inlineStr"/>
+      <c r="N39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Particles</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Deterministic varied explosions</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Use one seed and fire repeated explosive families at different materials</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Compare silhouettes ejecta smoke ember and debris then restart and repeat the sequence</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Explosions differ by event weapon and material but the exact repeated input sequence reproduces the same result</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Two matched captures and final hashes</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
+      <c r="M40" s="3" t="inlineStr"/>
+      <c r="N40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Anatomy</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Systemic limbs bleeding and blood reactions</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Use ballistic blunt explosive and heat damage against miners</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Observe part injury severing bleedout clotting cautery blood flow stains heat water and traction</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Vital destruction or bleedout kills; weapon classes affect parts differently; blood persists and reacts; and heat can cauterize bleeding</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Short capture plus event/debug notes</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
+      <c r="M41" s="3" t="inlineStr"/>
+      <c r="N41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Eight-voice stereo chip synthesis</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Use a stereo audio device and trigger overlapping fire hits blasts rope UI and bark events</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Listen for overlaps and compare two deterministic audio self-tests</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Original chip-style SFX use up to eight bounded voices with stereo placement; no music or samples play; and PCM hashes repeat</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Audio device description PCM hashes and capture</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr"/>
+      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr"/>
+      <c r="M42" s="3" t="inlineStr"/>
+      <c r="N42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Bots</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Perception and stateful AI</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Enable debug AI labels and play at least two seeds</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Hide break sight make noise damage a bot retreat and traverse a rope route</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Bots visibly transition among roaming searching attacking and retreating using LOS sound memory tools and terrain without reading hidden player state</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Seed state-transition notes and 60-second capture</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr"/>
+      <c r="K43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr"/>
+      <c r="M43" s="3" t="inlineStr"/>
+      <c r="N43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Miner Index navigation</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Open Miner Index from the title screen</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Move from first through last entry using only Up Down and Back</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Exactly six rows are visible; arrows indicate overflow; selection eases between rows; and the right one-page detail changes automatically for every unlocked entry</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>First middle and last-entry screenshots</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>How To Play one-pager</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Open How To Play with keyboard and controller</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Read the entire page and return with Back</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Movement rope combat objectives spawn shield and both input layouts fit on one readable page without scrolling</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Full-screen screenshot at default window size</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr"/>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
+      <c r="M45" s="3" t="inlineStr"/>
+      <c r="N45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Scripting</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Lua sandbox validation</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Build or use the script CLI</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Validate official DIGS sources then validate fixtures attempting os io package debug loadfile and an instruction-budget loop</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Official sources produce stable catalog hashes; forbidden capabilities and runaway scripts fail safely with readable diagnostics</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>CLI logs and source/catalog hashes</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr"/>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
+      <c r="M46" s="3" t="inlineStr"/>
+      <c r="N46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Scripting</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Transactional F5 reload</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Run a source checkout and make one valid then one invalid catalog edit</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Press F5 after each edit</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Valid data reloads with a new hash; invalid data reports an error and leaves the last valid catalog and running simulation intact</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Before-after hash and error screenshot</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr"/>
+      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr"/>
+      <c r="M47" s="3" t="inlineStr"/>
+      <c r="N47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Game Mode</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Miners versus Machines co-op</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Choose two humans Miners versus Machines and friendly fire Off then On</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Attack bots and each other under both settings</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Humans share a team objective; bot opponents remain fair; and human friendly damage follows the explicit toggle</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Setup screenshots and damage notes</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr"/>
+      <c r="N48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Controls</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard and controller rebinding</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Open Controls and rebind one movement one rope one fire and one weapon-cycle action</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Use the new bindings restart the match and then restore defaults</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Supported keyboard actions and controller buttons capture correctly; conflicts swap bindings; changes persist for the run; and restoring defaults works without affecting simulation determinism</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Controls screenshots and tested mapping list</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr"/>
+      <c r="K49" s="3" t="inlineStr"/>
+      <c r="L49" s="3" t="inlineStr"/>
+      <c r="M49" s="3" t="inlineStr"/>
+      <c r="N49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Combat UI</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Damage numbers and nonlocal health bars</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Damage one local and one bot fighter repeatedly</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Observe aggregates within 100 ms and wait without dealing damage</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Local-human damage events show bounded aggregated numbers with configured size/color; nonlocal health bars appear on damage then fade</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Short capture and setting values</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
+      <c r="M50" s="3" t="inlineStr"/>
+      <c r="N50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Two-controller claim and disconnect safety</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Connect two controllers and choose two local players</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Claim one controller per player; play simultaneously; disconnect either device</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Each device controls only its slot; simultaneous actions remain independent; and disconnect pauses before any slot is reassigned</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Controller IDs and short capture</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr"/>
+      <c r="K51" s="3" t="inlineStr"/>
+      <c r="L51" s="3" t="inlineStr"/>
+      <c r="M51" s="3" t="inlineStr"/>
+      <c r="N51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>FX Budget</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Retro Standard and Carnage profiles</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Run the same stress sequence under 768 1536 and 3072 budgets</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Monitor effect counts frame time and final authoritative state</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Each explicit simulation profile respects its selected cap and degrades safely; repeated runs with the same profile are deterministic; profile changes do not corrupt gameplay or crash</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Three debug captures benchmark notes and hashes</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr"/>
+      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr"/>
+      <c r="M52" s="3" t="inlineStr"/>
+      <c r="N52" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N32"/>
-  <conditionalFormatting sqref="H2:H32">
+  <autoFilter ref="A1:N52"/>
+  <conditionalFormatting sqref="H2:H52">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -2190,10 +3230,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3262,7 +4302,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Expected demo version is v0.0.1.</t>
+          <t>Expected demo version is v0.0.2.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: refine DIGS input maps and miner icon
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -582,22 +582,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Use the provided launch script or run digs_demo from a terminal</t>
+          <t>Use the DIGS! desktop shortcut or provided launch script</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Start the demo and wait for the title screen</t>
+          <t>Confirm the shortcut shows the pixel miner then start the demo and wait for the title screen</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The DIGS title screen appears without an error</t>
+          <t>The shortcut uses the exact in-game left-facing miner and the DIGS title screen appears without an error</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Build ID and a title-screen screenshot</t>
+          <t>Desktop and title-screen screenshots plus build ID</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -743,17 +743,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Start the match and inspect both sides of the arena</t>
+          <t>Traverse both sides and inspect seams drifts and overhead anchors</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The arena is playable and contains layered destructible terrain plus an intact bedrock boundary</t>
+          <t>The arena has broad rolling connected ground with exposed coal seams sand drifts sparse suspended rails and an intact bedrock boundary</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Seed and arena screenshot</t>
+          <t>Seed and full-arena screenshot</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Start the match and inspect caves and firedamp pockets</t>
+          <t>Enter the surface shafts and trace connected chambers firedamp pockets and natural anchors</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The arena is playable and exposes cave terrain with visible systemic material opportunities</t>
+          <t>The arena has connected chambers and surface-accessible vertical shafts with clustered firedamp and stone or coal rope routes</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Seed and arena screenshot</t>
+          <t>Seed and chamber-route screenshots</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -847,17 +847,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Start the match and inspect industrial terrain and sand</t>
+          <t>Traverse its terraces broken gantries open gaps and contained hot regions</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>The arena is playable and has a layout distinct from Coal Ridge and Deepworks</t>
+          <t>The industrial arena is structurally distinct with suspended gantries and limited heat or lava pockets but no surface-to-sky tower blocks the walk lane</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Seed and arena screenshot</t>
+          <t>Seed and full-arena screenshot</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Aim and fire at visible terrain from each local player at several frame caps</t>
+          <t>Switch P1 between mouse and controller aim then fire from each local player at several frame caps</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>The spring camera keeps both humans readable; action weighting remains stable; and each reticle debug target and impact agree</t>
+          <t>The spring camera keeps both humans readable; each player has exactly one active-source reticle; and every reticle debug target and impact agree</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Short capture plus zoom frame cap and impact location</t>
+          <t>Short capture plus input mode zoom frame cap and impact location</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -2241,27 +2241,27 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Controller hotplug and Xbox layout</t>
+          <t>Controller mapping raw fallback and hotplug</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Start with no controller then connect an Xbox-compatible controller</t>
+          <t>Start with no pad then connect a Logitech F310 in X mode and repeat in D mode</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Use the controller in menus and play; disconnect and reconnect it</t>
+          <t>Test menus movement radial aim weapon-aware reach calibration disconnect and reconnect in each mode</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>The controller is claimed once; all documented actions work; disconnect pauses safely; and reconnect allows reclaim</t>
+          <t>Known mappings and raw fallback each produce usable logical controls; noisy rest does not move aim; disconnect follows the selected AUTO or locked-mode safety behavior</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Controller model terminal output and short capture</t>
+          <t>Controller mode GUID SDL version input-setting values and short capture</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
@@ -2350,17 +2350,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Use visible beams arches and rock anchors</t>
+          <t>Use suspended rails gantries and natural rock anchors</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aim attach swing reel release and destroy the occupied anchor</t>
+          <t>Aim attach swing reel release cross the arena and destroy the occupied anchor</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Rope attaches only to stable solids; constrains distance; preserves release momentum; and detaches safely when the anchor breaks</t>
+          <t>Rope anchors remain within 30 cells; no support column blocks the walk lane; the rope preserves release momentum and detaches safely when its anchor breaks</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3021,27 +3021,27 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Keyboard and controller rebinding</t>
+          <t>Input modes tuning persistence and rebinding</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Open Controls and rebind one movement one rope one fire and one weapon-cycle action</t>
+          <t>Open Options then Input &amp; Controller and also open Controls</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Use the new bindings restart the match and then restore defaults</t>
+          <t>Cycle each P1 and P2 mode sensitivity deadzone and aim-slow setting; calibrate; rebind actions; relaunch; then restore defaults</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Supported keyboard actions and controller buttons capture correctly; conflicts swap bindings; changes persist for the run; and restoring defaults works without affecting simulation determinism</t>
+          <t>Settings persist safely; AUTO changes source only on deliberate input; locked modes ignore the other gameplay source; calibration and conflict swaps work; defaults restore without changing simulation determinism</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Controls screenshots and tested mapping list</t>
+          <t>Input and Controls screenshots settings file values and tested mapping list</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -3125,27 +3125,27 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Two-controller claim and disconnect safety</t>
+          <t>Exclusive two-player source ownership</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Connect two controllers and choose two local players</t>
+          <t>Connect zero one then two controllers and choose two local players</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Claim one controller per player; play simultaneously; disconnect either device</t>
+          <t>Exercise AUTO KEYBOARD and CONTROLLER modes while deliberately alternating sources and disconnecting either pad</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Each device controls only its slot; simultaneous actions remain independent; and disconnect pauses before any slot is reassigned</t>
+          <t>Every device owns at most one slot; idle sticks never steal keyboard input; one controller defaults to P2; two pads stay isolated; and source changes clear held fire jump and rope edges</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Controller IDs and short capture</t>
+          <t>Controller IDs selected modes and short capture</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: expand DIGS arenas and clear traversal
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -743,17 +743,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Traverse both sides and inspect seams drifts and overhead anchors</t>
+          <t>Traverse its land masses and inspect seams drifts and high anchors</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The arena has broad rolling connected ground with exposed coal seams sand drifts sparse suspended rails and an intact bedrock boundary</t>
+          <t>The arena has broad rolling ground with exposed coal seams sand drifts sparse high rope anchors and visible lava beyond safe land</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Seed and full-arena screenshot</t>
+          <t>Seed landform and full-arena screenshot</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1305,27 +1305,27 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Rising lava endgame</t>
+          <t>Visible basin and rising lava endgame</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Run a short test build or wait for the final 30 seconds of a classic match</t>
+          <t>Start a match then run a short test build or wait for the final 30 seconds</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Observe the bottom boundary and allow a miner to touch rising lava</t>
+          <t>Observe the initial lower boundary then allow a miner to touch lava before and during its rise</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Lava enters physical world cells; rises monotonically; and damages or kills a miner on contact</t>
+          <t>A real emissive lava basin is visible from match start; contact damages or kills; and the surface later rises monotonically through physical world cells</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Timed screenshots or capture and the debug tick</t>
+          <t>Initial and timed screenshots plus debug tick</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Shared dynamic zoom and aim alignment</t>
+          <t>Shared dynamic zoom aim and bounded framing</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2095,12 +2095,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Switch P1 between mouse and controller aim then fire from each local player at several frame caps</t>
+          <t>Switch P1 between mouse and controller aim then fire at several frame caps and pan toward every world edge</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>The spring camera keeps both humans readable; each player has exactly one active-source reticle; and every reticle debug target and impact agree</t>
+          <t>The spring camera keeps both humans readable; every reticle target and impact agree; and sky plus the lava horizon replace any would-be black exposure at every zoom and edge</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Ten-times mini-voxel profile</t>
+          <t>Forty-times mini-voxel profile</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2147,17 +2147,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Inspect terrain particles explosions and the occupied-cell count</t>
+          <t>Inspect terrain particles explosions world span and occupied-cell count</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>The demo uses a 256x160x10 world with granular terrain and effects at the denser scale</t>
+          <t>The demo uses a 512x320x10 world with 1638400 granular simulated cells while the CPU renderer remains responsive</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Screenshot seed occupied count and benchmark output</t>
+          <t>Screenshot seed occupied count memory note and benchmark output</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -2298,22 +2298,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Use a flat recorded seed and then rough terrain</t>
+          <t>Use a continent seed and then rough terrain</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Run reverse stop short-hop full-jump coyote jump-buffer and step-assist trials</t>
+          <t>Run reverse stop short-hop full-jump coyote jump-buffer and two-cell step-assist trials across a long route</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Acceleration is readable but responsive; reversal and stopping are precise; jump height responds to hold time; and small terrain steps do not dead-stop the miner</t>
+          <t>Acceleration is readable but responsive; reversal and stopping are precise; jump height responds to hold time; and density-scaled terrain steps do not dead-stop the miner</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Short capture with approximate flat-map traversal time</t>
+          <t>Short capture with approximate continent traversal time</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Deterministic breakable traversal rope</t>
+          <t>Deterministic high-anchor traversal rope</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aim attach swing reel release cross the arena and destroy the occupied anchor</t>
+          <t>Aim attach swing reel release across gaps and destroy the occupied anchor</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Rope anchors remain within 30 cells; no support column blocks the walk lane; the rope preserves release momentum and detaches safely when its anchor breaks</t>
+          <t>Rope anchors stay within 48 cells and 36 through 42 cells above nearby terrain; the lower 28 cells stay obstacle-free; release momentum and anchor destruction remain correct</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Seed anchor location and short capture</t>
+          <t>Seed anchor location clearance measurement and short capture</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -3216,9 +3216,113 @@
       <c r="M52" s="3" t="inlineStr"/>
       <c r="N52" s="3" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Landforms</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Archipelago continent and twin hills</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Use recorded seeds that select each macro landform while holding map style constant</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Zoom out inspect the full arena then traverse every reachable mass</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>The same material style produces three deterministic and visibly different macro layouts with useful sky safe terrain gaps edge drop-offs and exposed lava</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Three seeds and three full-arena screenshots</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr"/>
+      <c r="K53" s="3" t="inlineStr"/>
+      <c r="L53" s="3" t="inlineStr"/>
+      <c r="M53" s="3" t="inlineStr"/>
+      <c r="N53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Traversal</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Spawn floor and overhead clearance</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Start four-slot matches across all styles and landforms then jump beneath every generated metal anchor</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Record every spawn and test the complete jump envelope below fixtures</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Every fighter spawns on deep terrain rather than a suspended beam; no anchor boxes in a spawn or intersects the lower 28-cell traversal envelope</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Seed spawn coordinates and clearance captures</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr"/>
+      <c r="K54" s="3" t="inlineStr"/>
+      <c r="L54" s="3" t="inlineStr"/>
+      <c r="M54" s="3" t="inlineStr"/>
+      <c r="N54" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N52"/>
-  <conditionalFormatting sqref="H2:H52">
+  <autoFilter ref="A1:N54"/>
+  <conditionalFormatting sqref="H2:H54">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -3230,10 +3334,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H54" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I54" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: complete DIGS combat and audio feedback
Signed-off-by: claire-moon <cg@helloworldtwo.com>
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3320,9 +3320,633 @@
       <c r="M54" s="3" t="inlineStr"/>
       <c r="N54" s="3" t="inlineStr"/>
     </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Authoritative lava projection</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Start a match before the lava rise and move through every wheel zoom level</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Compare the lava surface at close zoom and overview zoom then pan until it is offscreen</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Only the true world-space lava horizon is drawn; zooming out reveals its actual position; close zoom has no fixed lava footer; and no camera edge exposes black</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Matched screenshots for every zoom plus seed and tick</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr"/>
+      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
+      <c r="M55" s="3" t="inlineStr"/>
+      <c r="N55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Weapons</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Projectile muzzle safety</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Stand in open space then near external walls and fire every projectile explosive</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Fire along all cardinal and diagonal aim directions then repeat a deliberate close-wall shot</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Projectiles clear the firing miner and launch envelope for six ticks; external walls still collide; and normal self-damage returns after clearance</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Short capture with weapon aim direction tick and damage result</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr"/>
+      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr"/>
+      <c r="M56" s="3" t="inlineStr"/>
+      <c r="N56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Match Rules</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Clock cap winner and draw</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Open Customize Game and test two and three minutes with score cap Off 5 10 and 20</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Reach time and score endings in FFA and Miners versus Machines including one exact tie</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>The full final tick resolves once; the correct individual or team wins; exact ties draw; and all active names scores deaths and end reason appear</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Setup and results screenshots plus final event notes</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr"/>
+      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr"/>
+      <c r="N57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-057</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Respawn</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>AUTO and ON FIRE timing</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Test delay values 0 1 2 3 and 5 under both respawn modes</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Die while holding Fire then release and press after readiness; repeat with a bot</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>AUTO returns at the selected delay; ON FIRE requires a fresh press; zero waits until the next step; bots return automatically; and the five-second shield remains</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Countdown captures with mode delay and debug ticks</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr"/>
+      <c r="K58" s="3" t="inlineStr"/>
+      <c r="L58" s="3" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr"/>
+      <c r="N58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-058</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Names editor and roster persistence</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Configure one and two human matches with bots and edit every active slot by keyboard and controller grid</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Use valid and invalid characters; relaunch; then complete a match</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Names are uppercase and limited to twelve supported characters; human names persist; bot names last one match; nameplates killfeed and results resolve the correct slots</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Editor setup gameplay and results screenshots plus sanitized values</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr"/>
+      <c r="K59" s="3" t="inlineStr"/>
+      <c r="L59" s="3" t="inlineStr"/>
+      <c r="M59" s="3" t="inlineStr"/>
+      <c r="N59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-059</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Combat Feedback</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Hit marker confirms and crosshair pulse</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Use each local human to damage and kill another miner while bots also fight</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Compare local hits local deaths and bot-only events under each Flash setting</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>A struck miner tints red; the impact marker and attacker crosshair pulse once; local hit and kill confirms sound; fullscreen flashes follow Options; bot-only events stay compact</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Short capture and audio or visual notes for P1 P2 and bots</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr"/>
+      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
+      <c r="M60" s="3" t="inlineStr"/>
+      <c r="N60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-060</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Awards</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Multikill and killing-spree chain</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Score kills inside and outside the three-second window then die after four uninterrupted kills and repeat to five</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Observe the feed banners and announcer for every boundary</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Two kills announce Double; three Triple; four or more Multi; five uninterrupted kills announce Killing Spree; expiry and death reset the correct counters</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Timed event log or capture with player names and ticks</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr"/>
+      <c r="K61" s="3" t="inlineStr"/>
+      <c r="L61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr"/>
+      <c r="N61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-061</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Menu motif zoom click and master volume</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Open every menu and Options then use mouse wheel zoom at each limit</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Navigate rapidly; wait more than 1.5 seconds; test Accept Back zoom Shift-wheel and master values 100 50 and 0</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Navigation walks the mining motif; idle resets it; only a successful unmodified wheel zoom clicks; Shift-wheel does not; and master zero is silent without stopping gameplay</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Audio capture settings values and input sequence</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr"/>
+      <c r="K62" s="3" t="inlineStr"/>
+      <c r="L62" s="3" t="inlineStr"/>
+      <c r="M62" s="3" t="inlineStr"/>
+      <c r="N62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-062</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Speech</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Announcer miner barks and bubbles</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Enter the title then start a match and trigger Bark with P1 C P2 M and controller R3</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Exercise six contexts and observe machines for at least sixty seconds</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>The deep voice announces title start and local awards; high miners speak matching bubbles; human speech is manual; and machine chatter stays sparse and non-tactical</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Audio-video capture with contexts controller and approximate bark times</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="inlineStr"/>
+      <c r="L63" s="3" t="inlineStr"/>
+      <c r="M63" s="3" t="inlineStr"/>
+      <c r="N63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-063</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Ambience</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>World-aware wind water and lava</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Visit open sky water and the lava basin at several camera zooms</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Hold the camera over each material then move between them during combat</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Smoothed procedural ambience follows visible world material and pan; at most two layers dominate; combat and speech remain readable; and hashes do not change</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Audio capture seed camera position and before-after hashes</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr"/>
+      <c r="N64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-064</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Schema migration and atomic recovery</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Back up the settings file then test schema 1 schema 2 an invalid file and a synthetic future schema</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Launch change one option exit and compare the file after each case</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Schema 1 migrates; schema 2 persists; invalid values fall back safely; a future schema is never overwritten; and a failed replacement retains the last readable file</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Before-after settings copies exit status and option screenshots</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr"/>
+      <c r="L65" s="3" t="inlineStr"/>
+      <c r="M65" s="3" t="inlineStr"/>
+      <c r="N65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-065</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Combat UI</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Stacked local death and award notices</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Use both local players to score chained kills that also cross the five-kill spree boundary</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Observe the centered notice rows killfeed audio and victim perspective</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Named kill context remains visible beside Double Triple Multi and Killing Spree awards; couch players are unambiguous; and no notice corrupts or hides the results state</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Short capture with active names kill ticks and visible notice rows</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr"/>
+      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N54"/>
-  <conditionalFormatting sqref="H2:H54">
+  <autoFilter ref="A1:N66"/>
+  <conditionalFormatting sqref="H2:H66">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -3334,10 +3958,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H54" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I54" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: deliver DIGS v0.0.3 stability systems
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$51</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="manual" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -3944,9 +3944,1205 @@
       <c r="M66" s="3" t="inlineStr"/>
       <c r="N66" s="3" t="inlineStr"/>
     </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-066</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Collision</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>No digging or collapse teleport</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Start a match with debug values visible and place a miner beside active sand stone and destructible support</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Dig blast and collapse terrain into the miner from several directions for at least two minutes</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>The miner moves only through ordinary velocity or a bounded local recovery; no living player silently jumps to a distant spawn and an impossible entombment produces one normal crush death</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Video with seed tick coordinates health deaths and event sequence</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr"/>
+      <c r="N67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-067</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Swept shots and visible anatomy</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Disable or wait out spawn protection and use nail gun shotgun melee blast and rail against each visible body region</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Fire across former two-cell sample gaps and at head torso arms hands pelvis legs and feet</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Every visible contact hits once at its actual location; clean misses and covered targets remain misses; each severable part has a visible result</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Slow capture with weapon impact marker anatomy and health</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr"/>
+      <c r="N68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-068</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Combat</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Spawn shield block feedback</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Attack a newly spawned miner with bullets blast melee rail and rope hook then repeat after five seconds</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Compare health velocity attribution markers sounds and events while protected and unprotected</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Protection preserves health anatomy velocity and attribution and emits distinct shield feedback; attacking still ends the owner's own shield</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Video and event/debug notes across all attack types</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr"/>
+      <c r="M69" s="3" t="inlineStr"/>
+      <c r="N69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-069</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Particles</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Natural debris without needle towers</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Detonate repeated explosives against one wall and kill miners above flat terrain</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Observe flesh blood rock smoke and loose debris until every particle lands or expires</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>TTL never creates a sky solid; impact deposits fall or disperse; no repeated same-column one-cell tower forms; living bodies are not filled with debris</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Before-after capture and final occupied or awake counts</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
+      <c r="M70" s="3" t="inlineStr"/>
+      <c r="N70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-070</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Rope</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Independent Hold and Toggle modes</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Set P1 rope to Hold and P2 to Toggle then reverse and relaunch</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Cast miss attach reel detach switch input sources die and respawn with each player</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Hold follows press and release; Toggle follows fresh presses; misses do not retry; source changes do not fake-release; death and new matches reset safely</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Settings copy plus two-player input capture</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr"/>
+      <c r="M71" s="3" t="inlineStr"/>
+      <c r="N71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-071</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Rope</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Hook hit exact one health rule</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Wait out shields and strike a full-health injured and one-health enemy with the casting hook then test a shielded target</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Inspect health anatomy score deaths attribution knockback and cable contact</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Every unshielded hook ends its cast and leaves the living target at exactly 1 HP with bounded knockback but no anatomy damage or score; shield blocks all effects; cable contact is harmless</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Event log and captures for every starting health</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr"/>
+      <c r="M72" s="3" t="inlineStr"/>
+      <c r="N72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-072</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Rope</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Stable wrapping swing and anchors</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Use terrain corners gantries ceilings and destructible natural anchors</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Cast around corners swing reel unwrap reverse direction and destroy the anchor</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>The segmented rope wraps and unwraps predictably without snag explosions or stored-energy launch; reel and momentum remain controllable; destroyed or unstable anchors break once</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Traversal capture with tension and coordinates</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr"/>
+      <c r="L73" s="3" t="inlineStr"/>
+      <c r="M73" s="3" t="inlineStr"/>
+      <c r="N73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-073</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Weapons</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Charged energy-piercing Mining Rail</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Use Full Works and direct-select the Mining Rail with minus or cycle input</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Tap and fully charge shots through soft terrain aligned miners stone and bedrock</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Charge tell release beam four-tick afterimage recoil cooldown sound and haptics agree; energy decreases through bodies and soft material; strong stone or bedrock stops it; full vital hit is lethal</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Video with charge ticks impacts damage and material path</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="inlineStr"/>
+      <c r="M74" s="3" t="inlineStr"/>
+      <c r="N74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-074</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Lift-and-glide steampack</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Use keyboard and controller on open terrain slopes gaps and under ceilings</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Apply short pulses full burns direction reversals and release glides until fuel empties then recharge</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Thrust is controllable and capped; lateral steering and opposite-input braking are accurate; momentum carries naturally; collision remains stable; small lit pack flame and exhaust track actual thrust without affecting terrain</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Trajectory capture with fuel velocity and frame cap</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr"/>
+      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
+      <c r="M75" s="3" t="inlineStr"/>
+      <c r="N75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-075</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Qualified 15 through Unlimited caps</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Run startup qualification and inspect every frame-cap choice on the test machine</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>Select each supported cap and run movement explosion rope and rail scenes for two minutes</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Unsupported caps are visibly gated instead of pretending; supported caps meet their deadlines while authoritative simulation stays at 60 Hz with no tick-debt loss</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Qualification result debug frametime and state hashes</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr"/>
+      <c r="N76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-076</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Laptop Mode presentation parity</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Record a seed and input sequence then run it once with Laptop Mode Off and once On</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>Compare movement bots particles damage terrain clock and final hash while observing render quality</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Authoritative rules FX budget particle simulation bot decisions material results and final hash match exactly; only cached or reduced presentation work differs</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Labeled captures settings and matching final hashes</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
+      <c r="M77" s="3" t="inlineStr"/>
+      <c r="N77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-077</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Frame-independent device-clock sound</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Run the same menu speech ambience weapon and combo sequence at 15 30 60 144 and Unlimited</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Record output duration pitch cadence and any dropout while forcing an irregular render load</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Sound duration pitch and sequencing remain stable without underruns or repeated frame-linked beeps; silence fallback never changes gameplay</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Audio recordings frame caps callback diagnostics and hashes</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
+      <c r="M78" s="3" t="inlineStr"/>
+      <c r="N78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Switch Pro USB controls and prompts</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Connect a Nintendo Switch Pro Controller by USB before launch then repeat hotplug and calibration</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>Use menus movement aim zoom rope rail bark and pause while inspecting every shown prompt</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Nintendo A B X Y L R ZL ZR Plus Minus and stick labels match physical controls; no duplicate crosshair appears; standard rumble works or reports a graceful driver limitation</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Controller GUID connection path screenshots and capture</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
+      <c r="M79" s="3" t="inlineStr"/>
+      <c r="N79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-079</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Switch Pro Bluetooth controls and prompts</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Pair a Nintendo Switch Pro Controller over Bluetooth before launch then repeat reconnect during menus and play</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Use the complete USB checkpoint sequence and compare mappings haptics disconnect and reclaim</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Nintendo labels and actions match the USB layout; disconnect is safe; reclaim is deterministic; available rumble works without stuck motors</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Controller GUID Bluetooth stack screenshots and capture</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr"/>
+      <c r="K80" s="3" t="inlineStr"/>
+      <c r="L80" s="3" t="inlineStr"/>
+      <c r="M80" s="3" t="inlineStr"/>
+      <c r="N80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-080</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Haptics</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Local distance-weighted vibration levels</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Use two controllers and cycle Off Low Normal and Heavy while firing moving by collapse taking hits killing and observing distant bot fights</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Compare motor strength duration locality and simultaneous-event behavior for both local players</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Every level is distinct; Off is silent; own fire rope hits nearby explosions kills and crumble differ; distance attenuates world events; distant bot-only events do not vibrate locals; no envelope sticks</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Two-controller event list and video or tester notes</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr"/>
+      <c r="K81" s="3" t="inlineStr"/>
+      <c r="L81" s="3" t="inlineStr"/>
+      <c r="M81" s="3" t="inlineStr"/>
+      <c r="N81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-081</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Console-appropriate active-source glyphs</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Connect Nintendo Xbox PlayStation and generic controllers when available and alternate each with keyboard</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Inspect title menus setup Controls Options index pause and gameplay prompts after rebinds and source changes</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Prompts follow the active player's actual binding and controller family with correct face shoulder trigger menu and stick labels; generic fallback stays readable</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Per-device IDs prompt screenshots and rebound mapping</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr"/>
+      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
+      <c r="M82" s="3" t="inlineStr"/>
+      <c r="N82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-082</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Controller zoom and close voxel detail</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Use one-human bot play then a two-human shared-camera match</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>Hold ZL or left trigger and move the right stick vertically through all zooms; compare close voxels lighting HUD lava and edge framing</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Controller and mouse zoom agree; close view reveals native adjacent voxels and Lightfield detail while HUD stays on its pixel grid; only the visible shared-camera region renders; no black or scaled lava appears</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Screenshots at every zoom with frame timing and player count</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr"/>
+      <c r="K83" s="3" t="inlineStr"/>
+      <c r="L83" s="3" t="inlineStr"/>
+      <c r="M83" s="3" t="inlineStr"/>
+      <c r="N83" s="3" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-083</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Speech</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Context library names and Dummy Mode</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Set distinctive player names and trigger barks during roaming search attack retreat hurt kill low health rope lava fire digging and material discovery</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Repeat with Dummy Mode Off and On then observe bots for two minutes</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Lines vary through curated and seeded pools; names weapons materials and hazards are relevant; unknown names pronounce or spell deterministically; Off enforces three seconds; Dummy permits local spam only; bots remain sparse</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Transcript seed names contexts timings and audio-video capture</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr"/>
+      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
+      <c r="M84" s="3" t="inlineStr"/>
+      <c r="N84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-084</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Two-human two-bot destruction soak</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Run a four-slot Full Works match with Carnage FX rising lava repeated explosives rail rope and barks</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Play for fifteen minutes while recording simulation average p95 maximum awake cells audio callbacks render deadlines and final state</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>No crash teleport tower audio underrun tick-debt loss or controller crossover occurs; named test-bench simulation meets 5 ms average 8 ms p95 and 16.67 ms maximum</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Raw timing log settings seed final hash and cockpit packet</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr"/>
+      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
+      <c r="M85" s="3" t="inlineStr"/>
+      <c r="N85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-085</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Anatomy</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Dismemberment gameplay verification</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Wait out shields and use ballistic explosive melee heat rail and bleed paths against every anatomy region</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Observe health bleeding cautery severed visuals death attribution gore and legitimate respawn reset</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Real contacts drive exact anatomy; every severable part visibly changes; vital and bleed deaths score once with the damaging weapon; only a legitimate respawn restores anatomy</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Annotated captures event log weapon path and before-after anatomy</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr"/>
+      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
+      <c r="M86" s="3" t="inlineStr"/>
+      <c r="N86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-086</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Haptic mixer isolation self-test</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Use the exact v0.0.3 digs_demo binary</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Run digs_demo --haptic-self-test</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>The command exits zero; Off is zero; Low is less than Normal; Normal is less than Heavy; Near is greater than Far; and the values repeat for the same build</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Self-test log binary SHA-256 and exit status; physical controller rumble remains Not Run</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr"/>
+      <c r="K87" s="3" t="inlineStr"/>
+      <c r="L87" s="3" t="inlineStr"/>
+      <c r="M87" s="3" t="inlineStr"/>
+      <c r="N87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-087</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Portable four-slot 600-tick load regression</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Use the exact v0.0.3 digs_demo binary on any supported SDL2 host</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Run digs_demo --load-self-test 600</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>The command exits zero with ticks 600 slots 4 local 2 bots 2 fired 46 explosions 26 crushes 0 effects 700 awake 7867 and hash f3924b81; no wall-clock threshold is applied</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Complete load self-test log binary SHA-256 platform and exit status</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr"/>
+      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
+      <c r="M88" s="3" t="inlineStr"/>
+      <c r="N88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-088</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Named-laptop 600-tick performance qualification</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Use the i7-10750H GTX 1660 Ti laptop bench in power-saver; close unrelated heavy work and record exact binary</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Run digs_demo --performance-self-test 600 or package with VOX_NAMED_BENCH_QUALIFY=1</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>The command exits zero with canonical 600-tick activity and hash; average is at most 5 ms; p95 is at most 8 ms; maximum is at most 16.67 ms; shared hosted runner timing cannot pass this checkpoint</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Complete qualification log binary SHA-256 CPU power profile temperatures and exit status</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr"/>
+      <c r="K89" s="3" t="inlineStr"/>
+      <c r="L89" s="3" t="inlineStr"/>
+      <c r="M89" s="3" t="inlineStr"/>
+      <c r="N89" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N66"/>
-  <conditionalFormatting sqref="H2:H66">
+  <autoFilter ref="A1:N89"/>
+  <conditionalFormatting sqref="H2:H89">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -3958,10 +5154,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H89" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I89" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4949,7 +6145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -5030,7 +6226,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Expected demo version is v0.0.2.</t>
+          <t>Expected demo version is v0.0.3.</t>
         </is>
       </c>
     </row>
@@ -5307,133 +6503,133 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Frame caps tested</t>
+          <t>Test lane</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>VOX Options</t>
+          <t>Manual</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>List 30 60 90 120 144 and Unlimited as tested.</t>
+          <t>Quick Full Automation Build-only or another clearly named lane.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Lightfield tiers tested</t>
+          <t>QA run ID</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>VOX Options</t>
+          <t>Cockpit or manual</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>List Compatibility Balanced and Showcase.</t>
+          <t>Use the cockpit run ID when available.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Input devices</t>
+          <t>Frame caps tested</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>VOX Options</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Keyboard and pointing device model or type.</t>
+          <t>List 15 30 60 90 120 144 and Unlimited as tested.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Audio device</t>
+          <t>Cap qualification result</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>System settings</t>
+          <t>VOX startup / self-test</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Use a general device label; omit unique IDs.</t>
+          <t>List supported and visibly gated caps; do not infer support.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Power state</t>
+          <t>Lightfield tiers tested</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>VOX Options</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>AC or battery and relevant performance profile.</t>
+          <t>List Compatibility Balanced and Showcase.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>xleak version</t>
+          <t>Laptop Mode</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>xleak --version</t>
+          <t>VOX Options</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Cockpit dependency version.</t>
+          <t>Record Off or On for every parity/hash run.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Test started UTC</t>
+          <t>Dummy Mode</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Manual</t>
+          <t>VOX Options</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Use ISO 8601: YYYY-MM-DDTHH:MM:SSZ.</t>
+          <t>Record Off or On for bark-cooldown evidence.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Test ended UTC</t>
+          <t>Input devices</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr"/>
@@ -5444,32 +6640,446 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Use ISO 8601: YYYY-MM-DDTHH:MM:SSZ.</t>
+          <t>Keyboard and pointing device model or type.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Evidence sharing consent</t>
+          <t>Controller model / SDL name</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
+          <t>SDL / manual</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>General model/name only; omit unique serial data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Controller SDL GUID</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>SDL diagnostics</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Controller mapping identity; never substitute a hardware serial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Controller transport</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Record USB Bluetooth or other without unique serial data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Controller prompt family</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>VOX UI</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Record Nintendo Xbox PlayStation or generic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Controller mapping path</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>VOX diagnostics</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Record SDL mapped or raw joystick fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>P1 / P2 input ownership</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>VOX Options</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Record AUTO KEYBOARD CONTROLLER and claimed pad per local player.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Aim calibration</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>VOX Options</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Record sensitivity deadzone aim slowdown and whether calibration ran.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>P1 / P2 rope mode</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>VOX Options</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Record Hold or Toggle independently for each local player.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Haptics level / availability</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>VOX Options / SDL</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Record Off Low Normal Heavy and available blocked or unsupported.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Haptic mixer self-test result</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>VOX automation log</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Record off low normal heavy near and far values; this does not prove physical rumble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Audio device</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>System settings</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Use a general device label; omit unique IDs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Audio backend / cadence result</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>SDL / VOX self-test</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Record backend and callback underrun or cadence result when exposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Power state</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>AC or battery and relevant performance profile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Map style / landform / seed</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Match setup</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Required for terrain collision debris and camera reproduction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Local players / bots</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Match setup</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Record the active slot composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>FX profile</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Match setup</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Record Retro Standard or Carnage for simulation/hash comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Deterministic load self-test result</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>VOX automation log</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Record the 600-tick slots activity awake cells canonical hash and exit status; no timing threshold applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Named-bench performance qualification</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>VOX automation log</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Record average p95 maximum activity hash and power profile only from the named i7-10750H laptop bench.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Initial / final state hash</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>F1 / automation log</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Record both when comparing caps or Laptop Mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Frame hash / smoke SHA-256</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Automation log</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Identifies deterministic presentation evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>xleak version</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>xleak --version</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Cockpit dependency version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Test started UTC</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Use ISO 8601: YYYY-MM-DDTHH:MM:SSZ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Test ended UTC</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Use ISO 8601: YYYY-MM-DDTHH:MM:SSZ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Evidence sharing consent</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr"/>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Enter Yes only after reviewing the privacy checklist.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D28"/>
+  <autoFilter ref="A1:D51"/>
   <dataValidations count="1">
-    <dataValidation sqref="B28" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Confirm only after reviewing qa/README.md." type="list" errorStyle="stop">
+    <dataValidation sqref="B51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Confirm only after reviewing qa/README.md." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
build(release): establish v005 package foundation
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -4061,22 +4061,22 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Independent Hold and Toggle modes</t>
+          <t>Always-toggle Steam Hook and cancel</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Set P1 rope to Hold and P2 to Toggle then reverse and relaunch</t>
+          <t>Use one or two local players with the default current bindings</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Cast miss attach reel detach switch input sources die and respawn with each player</t>
+          <t>Cast miss attach reel retarget with a second press jump-cancel switch input sources die and respawn with each player</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Hold follows press and release; Toggle follows fresh presses; misses do not retry; source changes do not fake-release; death and new matches reset safely</t>
+          <t>A press casts or attaches; the next press retargets; jump cancels; misses do not retry; source changes do not fake-release; death and new matches reset safely</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -5309,7 +5309,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Saved history stays out of the match hash</t>
+          <t>Wall-clock metadata stays out of the match hash</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -5324,12 +5324,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Both print the same canonical state hash regardless of how much history each has accumulated; the saved layer is versioned and never enters the authoritative simulation</t>
+          <t>The controlled load self-test prints the same canonical state hash because it opens from a canonical snapshot; a real match opened from carried memory may differ as intended; no wall-clock metadata changes either result</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Both complete self-test logs and the two chronicle files</t>
+          <t>Both complete load self-test logs the two chronicle files and a cross-session evidence result</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Expected demo version is v0.0.4.</t>
+          <t>Expected demo version is v0.0.5.</t>
         </is>
       </c>
     </row>
@@ -7501,18 +7501,18 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>P1 / P2 rope mode</t>
+          <t>P1 / P2 grapple behavior</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>VOX Options</t>
+          <t>VOX Controls</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Record Hold or Toggle independently for each local player.</t>
+          <t>Record the always-toggle binding plus tested retarget and jump-cancel paths.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(qa): refresh feedback workbook
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Deterministic high-anchor traversal rope</t>
+          <t>Deterministic fixture-anchor traversal rope</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aim attach swing reel release across gaps and destroy the occupied anchor</t>
+          <t>Aim attach swing reel release across gaps then destroy an authored metal fixture and blast nearby terrain</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Rope anchors stay within 48 cells and 36 through 42 cells above nearby terrain; the lower 28 cells stay obstacle-free; release momentum and anchor destruction remain correct</t>
+          <t>Fixtures stay static solid rope targets until destroyed; a destroyed fixture detaches once and never becomes a new anchor; nearby real terrain may collapse independently</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Seed anchor location clearance measurement and short capture</t>
+          <t>Seed anchor location clearance measurement alert state and short capture</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -4009,27 +4009,27 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Natural debris without needle towers</t>
+          <t>Material fragments and impact-only gore</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Detonate repeated explosives against one wall and kill miners above flat terrain</t>
+          <t>Detonate repeated explosives against one wall then use pick and Railshot on soil stone coal sand and metal; kill miners above flat terrain</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Observe flesh blood rock smoke and loose debris until every particle lands or expires</t>
+          <t>Observe source-material fragments through flight bounce loose settling and gore through terrain impact</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>TTL never creates a sky solid; impact deposits fall or disperse; no repeated same-column one-cell tower forms; living bodies are not filled with debris</t>
+          <t>Player-cut terrain flies as real material then restores only as loose nonblocking terrain; fragments stay behind and pass through miners; blood stains only a struck surface; no airborne expiry tower or player blockage occurs</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Before-after capture and final occupied or awake counts</t>
+          <t>Before-after capture seed weapon tick final terrain and miner state</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>The binary plus the staged share tree is at or below 1474560 bytes; the report prints the measured payload and the percentage of the ceiling; documentation and evidence are excluded from the budget</t>
+          <t>The binary plus the staged share tree is at or below 10485760 bytes; the report prints the measured payload and the percentage of the ceiling; documentation and evidence are excluded from the budget</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(digs): stabilize fixtures and terrain fragments (#11)
* fix(digs): stabilize fixtures and terrain fragments

* chore(qa): refresh feedback workbook

* fix(digs): lock fixture and remnant stability

* fix(release): close package and API audit gaps

---------

Co-authored-by: AGENT-002 <agent-002@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Deterministic high-anchor traversal rope</t>
+          <t>Deterministic fixture-anchor traversal rope</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2355,17 +2355,17 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Aim attach swing reel release across gaps and destroy the occupied anchor</t>
+          <t>Aim attach swing reel release across gaps then destroy an authored metal fixture and blast nearby terrain</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Rope anchors stay within 48 cells and 36 through 42 cells above nearby terrain; the lower 28 cells stay obstacle-free; release momentum and anchor destruction remain correct</t>
+          <t>Fixtures stay static solid rope targets until destroyed; their moving scrap never becomes a replacement fixture anchor; any later settled ordinary metal follows normal terrain behavior; nearby real terrain may collapse independently</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Seed anchor location clearance measurement and short capture</t>
+          <t>Seed anchor location clearance measurement alert state and short capture</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -4009,27 +4009,27 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Natural debris without needle towers</t>
+          <t>Material fragments and impact-only gore</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Detonate repeated explosives against one wall and kill miners above flat terrain</t>
+          <t>Detonate repeated explosives against one wall then use pick and Railshot on soil stone coal sand and metal; kill miners above flat terrain</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Observe flesh blood rock smoke and loose debris until every particle lands or expires</t>
+          <t>Observe source-material fragments through flight bounce loose settling and gore through terrain impact</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>TTL never creates a sky solid; impact deposits fall or disperse; no repeated same-column one-cell tower forms; living bodies are not filled with debris</t>
+          <t>Player-cut terrain flies as real material then restores only as loose nonblocking terrain; fragments stay behind and pass through miners; blood stains only a struck surface; no airborne expiry tower or player blockage occurs</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Before-after capture and final occupied or awake counts</t>
+          <t>Before-after capture seed weapon tick final terrain and miner state</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>The binary plus the staged share tree is at or below 1474560 bytes; the report prints the measured payload and the percentage of the ceiling; documentation and evidence are excluded from the budget</t>
+          <t>The binary plus the staged share tree is at or below 10485760 bytes; the report prints the measured payload and the percentage of the ceiling; documentation and evidence are excluded from the budget</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">

</xml_diff>